<commit_message>
Fix Excel import-template dropdowns so they show in desktop Excel.
Point lists at a visible sheet with direct cell ranges, and drop the hidden-sheet named ranges and comments that made Excel repair the file and strip validation.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/frontend/campaign-import-template.xlsx
+++ b/frontend/campaign-import-template.xlsx
@@ -8,26 +8,25 @@
   </bookViews>
   <sheets>
     <sheet name="Import" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Lists" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet name="DropdownLists" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="How to fill" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="Webinar">Lists!$G$2:$G$2</definedName>
-    <definedName name="Event">Lists!$H$2:$H$8</definedName>
-    <definedName name="Email">Lists!$I$2:$I$3</definedName>
-    <definedName name="Paid">Lists!$J$2:$J$4</definedName>
-    <definedName name="Organic">Lists!$K$2:$K$3</definedName>
-    <definedName name="Content_Syndication">Lists!$L$2:$L$2</definedName>
-    <definedName name="Website_Gated">Lists!$M$2:$M$2</definedName>
-    <definedName name="Referral">Lists!$N$2:$N$2</definedName>
-    <definedName name="Direct_Mail">Lists!$O$2:$O$2</definedName>
-    <definedName name="CampaignTypeList">Lists!$A$2:$A$10</definedName>
-    <definedName name="TypeList">Lists!$B$2:$B$4</definedName>
-    <definedName name="ActionList">Lists!$C$2:$C$4</definedName>
-    <definedName name="Asset">Lists!$D$2:$D$40</definedName>
-    <definedName name="Tactic">Lists!$E$2:$E$32</definedName>
-    <definedName name="Campaign">Lists!$F$2:$F$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Import'!$A$1:$BN$1</definedName>
+    <definedName name="Webinar">DropdownLists!$G$2:$G$2</definedName>
+    <definedName name="Event">DropdownLists!$H$2:$H$8</definedName>
+    <definedName name="Email">DropdownLists!$I$2:$I$3</definedName>
+    <definedName name="Paid">DropdownLists!$J$2:$J$4</definedName>
+    <definedName name="Organic">DropdownLists!$K$2:$K$3</definedName>
+    <definedName name="Content_Syndication">DropdownLists!$L$2:$L$2</definedName>
+    <definedName name="Website_Gated">DropdownLists!$M$2:$M$2</definedName>
+    <definedName name="Referral">DropdownLists!$N$2:$N$2</definedName>
+    <definedName name="Direct_Mail">DropdownLists!$O$2:$O$2</definedName>
+    <definedName name="CampaignTypeList">DropdownLists!$A$2:$A$10</definedName>
+    <definedName name="TypeList">DropdownLists!$B$2:$B$4</definedName>
+    <definedName name="ActionList">DropdownLists!$C$2:$C$4</definedName>
+    <definedName name="Asset">DropdownLists!$D$2:$D$40</definedName>
+    <definedName name="Tactic">DropdownLists!$E$2:$E$32</definedName>
+    <definedName name="Campaign">DropdownLists!$F$2:$F$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -175,26 +174,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Budget app</author>
-  </authors>
-  <commentList>
-    <comment ref="F1" authorId="0" shapeId="0">
-      <text>
-        <t>Fill CampaignType first. SubCampaignType dropdown then shows only matching values.</t>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <t>For Type=Asset or Type=Tactic rows. Campaign rows leave LineName blank.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1158,37 +1137,53 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:BN1"/>
   <dataValidations count="5">
     <dataValidation sqref="A2:A500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Pick Create, Update, or Delete" promptTitle="Choose from list" prompt="Create, Update, or Delete" type="list">
-      <formula1>=ActionList</formula1>
+      <formula1>=DropdownLists!$C$2:$C$4</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Pick a campaign type from the list" promptTitle="Choose from list" prompt="Pick a campaign type first" type="list">
-      <formula1>=CampaignTypeList</formula1>
+      <formula1>=DropdownLists!$A$2:$A$10</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="That sub type does not belong to the selected campaign type" promptTitle="Choose from list" prompt="Pick a campaign type in this row first, then a matching sub type" type="list">
+    <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="That sub type does not belong to the selected campaign type" promptTitle="Choose from list" prompt="Pick CampaignType in this row first, then a matching sub type" type="list">
       <formula1>=INDIRECT(SUBSTITUTE($F2," ","_"))</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Pick Campaign, Asset, or Tactic" promptTitle="Choose from list" prompt="Campaign (metadata), Asset, or Tactic (spend line)" type="list">
-      <formula1>=TypeList</formula1>
+      <formula1>=DropdownLists!$B$2:$B$4</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="LineName must match the Type (Asset list or Tactic list)" promptTitle="Choose from list" prompt="Set Type to Asset or Tactic, then pick LineName" type="list">
       <formula1>=INDIRECT($H2)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001584A6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
+    <col width="28" customWidth="1" min="14" max="14"/>
+    <col width="28" customWidth="1" min="15" max="15"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1293,7 +1288,11 @@
           <t>AE Emails</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>(leave LineName blank)</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>Webinar</t>
@@ -1877,7 +1876,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1890,18 +1889,20 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="160" customHeight="1">
+    <row r="3" ht="200" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>1. Keep the Import sheet headers as they are.
+          <t>Open this file in Microsoft Excel (desktop). Google Sheets, Excel for the web, and Apple Numbers often ignore these dropdowns.
+1. Keep the Import sheet headers as they are.
 2. One Type=Campaign row per campaign (Team, Campaign, CampaignType, SubCampaignType, …).
 3. Then one Type=Asset or Type=Tactic row per spend line. Rows link by Campaign name.
 4. Pick CampaignType first — SubCampaignType then only shows related values.
 5. Pick Type = Asset or Tactic — LineName then only shows that list.
 6. Leave LineName blank on Campaign rows.
 7. Delete the example rows before importing real data.
-8. Upload this .xlsx (or Save As CSV) in Data Entry → Bulk import.
-9. Values are saved as the same text fields as the campaign form — no extra database columns.</t>
+8. Upload this .xlsx in Data Entry → Bulk import.
+9. Do not delete the DropdownLists sheet — the dropdowns read from it.
+10. Values are saved as the same text fields as the campaign form.</t>
         </is>
       </c>
     </row>
@@ -1914,9 +1915,11 @@
     <row r="10"/>
     <row r="11"/>
     <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A3:A12"/>
+    <mergeCell ref="A3:A14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Make campaign import dropdowns work in Google Sheets.
Use simple list ranges instead of INDIRECT so Sheets keeps the arrows; import still rejects mismatched subtype and LineName pairs.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/frontend/campaign-import-template.xlsx
+++ b/frontend/campaign-import-template.xlsx
@@ -11,23 +11,7 @@
     <sheet name="DropdownLists" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="How to fill" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames>
-    <definedName name="Webinar">DropdownLists!$G$2:$G$2</definedName>
-    <definedName name="Event">DropdownLists!$H$2:$H$8</definedName>
-    <definedName name="Email">DropdownLists!$I$2:$I$3</definedName>
-    <definedName name="Paid">DropdownLists!$J$2:$J$4</definedName>
-    <definedName name="Organic">DropdownLists!$K$2:$K$3</definedName>
-    <definedName name="Content_Syndication">DropdownLists!$L$2:$L$2</definedName>
-    <definedName name="Website_Gated">DropdownLists!$M$2:$M$2</definedName>
-    <definedName name="Referral">DropdownLists!$N$2:$N$2</definedName>
-    <definedName name="Direct_Mail">DropdownLists!$O$2:$O$2</definedName>
-    <definedName name="CampaignTypeList">DropdownLists!$A$2:$A$10</definedName>
-    <definedName name="TypeList">DropdownLists!$B$2:$B$4</definedName>
-    <definedName name="ActionList">DropdownLists!$C$2:$C$4</definedName>
-    <definedName name="Asset">DropdownLists!$D$2:$D$40</definedName>
-    <definedName name="Tactic">DropdownLists!$E$2:$E$32</definedName>
-    <definedName name="Campaign">DropdownLists!$F$2:$F$2</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -35,13 +19,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -91,12 +78,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1141,17 +1129,17 @@
     <dataValidation sqref="A2:A500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Pick Create, Update, or Delete" promptTitle="Choose from list" prompt="Create, Update, or Delete" type="list">
       <formula1>=DropdownLists!$C$2:$C$4</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Pick a campaign type from the list" promptTitle="Choose from list" prompt="Pick a campaign type first" type="list">
+    <dataValidation sqref="F2:F500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Pick a campaign type from the list" promptTitle="Choose from list" prompt="Pick a campaign type" type="list">
       <formula1>=DropdownLists!$A$2:$A$10</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="That sub type does not belong to the selected campaign type" promptTitle="Choose from list" prompt="Pick CampaignType in this row first, then a matching sub type" type="list">
-      <formula1>=INDIRECT(SUBSTITUTE($F2," ","_"))</formula1>
+    <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Pick a sub type from the list" promptTitle="Choose from list" prompt="Must match the CampaignType on this row (checked on import)" type="list">
+      <formula1>=DropdownLists!$D$2:$D$20</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Pick Campaign, Asset, or Tactic" promptTitle="Choose from list" prompt="Campaign (metadata), Asset, or Tactic (spend line)" type="list">
       <formula1>=DropdownLists!$B$2:$B$4</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="LineName must match the Type (Asset list or Tactic list)" promptTitle="Choose from list" prompt="Set Type to Asset or Tactic, then pick LineName" type="list">
-      <formula1>=INDIRECT($H2)</formula1>
+    <dataValidation sqref="I2:I500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Pick a LineName from the list" promptTitle="Choose from list" prompt="Assets and tactics. Import rejects a name that does not match Type." type="list">
+      <formula1>=DropdownLists!$E$2:$E$67</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1165,7 +1153,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O40"/>
+  <dimension ref="A1:E67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1173,92 +1161,32 @@
     <col width="28" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="28" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
-    <col width="28" customWidth="1" min="12" max="12"/>
-    <col width="28" customWidth="1" min="13" max="13"/>
-    <col width="28" customWidth="1" min="14" max="14"/>
-    <col width="28" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>CampaignType</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Asset</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Tactic</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Campaign</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Webinar</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Event</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Paid</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Organic</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Content Syndication</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Website Gated</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>Referral</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>Direct Mail</t>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>SubCampaignType</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>LineName</t>
         </is>
       </c>
     </row>
@@ -1280,62 +1208,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>Webinar</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>1:1 Meeting</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>AE Emails</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>(leave LineName blank)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Webinar</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Virtual Event</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Email Campaign</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Paid Search</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Organic Social</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Content Syndication</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Demo Request</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Referral Traffic</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>Direct Mail</t>
         </is>
       </c>
     </row>
@@ -1357,32 +1235,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>Virtual Event</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>Agency Retainer</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Agency Retainer</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>In-Person Event</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Nurture Campaign</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Paid Social</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Organic Search</t>
         </is>
       </c>
     </row>
@@ -1404,22 +1262,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>In-Person Event</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>Battle Cards</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Chat</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Executive Dinner</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Display</t>
         </is>
       </c>
     </row>
@@ -1431,17 +1279,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>Executive Dinner</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>Blog</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Content Syndication</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Workshop</t>
         </is>
       </c>
     </row>
@@ -1453,17 +1296,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
+          <t>Workshop</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>Booth</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Customer Retention &amp; Growth</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Customer Event</t>
         </is>
       </c>
     </row>
@@ -1475,17 +1313,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
+          <t>Customer Event</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
           <t>Case Studies</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Direct Mails</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Partner Event</t>
         </is>
       </c>
     </row>
@@ -1497,17 +1330,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
+          <t>Partner Event</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
           <t>Contact Request</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Direct Traffic</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Third-Party Event</t>
         </is>
       </c>
     </row>
@@ -1519,12 +1347,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
+          <t>Third-Party Event</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
           <t>Demand Gen Page</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Display</t>
         </is>
       </c>
     </row>
@@ -1536,332 +1364,461 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
+          <t>Email Campaign</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
           <t>eBook</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>External List Buys</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="D11" t="inlineStr">
         <is>
+          <t>Nurture Campaign</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
           <t>Employment Guide</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>In-Product</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="D12" t="inlineStr">
         <is>
+          <t>Paid Search</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
           <t>Event Registrations</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Influencer</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="D13" t="inlineStr">
         <is>
+          <t>Paid Social</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
           <t>Event Sponsorship</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Internal Referral</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="D14" t="inlineStr">
         <is>
+          <t>Display</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
           <t>Goodies/Swag</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Marketing Emails</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="D15" t="inlineStr">
         <is>
+          <t>Organic Social</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
           <t>Guide</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Newsletter</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="D16" t="inlineStr">
         <is>
+          <t>Organic Search</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
           <t>Infographics</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Organic Search</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="D17" t="inlineStr">
         <is>
+          <t>Content Syndication</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
           <t>Inquiry</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Organic Social</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="D18" t="inlineStr">
         <is>
+          <t>Demo Request</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
           <t>Interactive Asset</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Outbound Prospecting</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="D19" t="inlineStr">
         <is>
+          <t>Referral Traffic</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
           <t>Interactive Demos</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Paid Search</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="D20" t="inlineStr">
         <is>
+          <t>Direct Mail</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
           <t>Landing Page Copy</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+    </row>
+    <row r="21">
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Marketing Emails</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Marketplace Signups</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>On-Demand Webinar</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Other Miscellaneous</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Partner Lead Submission</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Presentation</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Promotion fee for ISV/Channel Partner</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>ROI Calculator</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Survey</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Translations &amp; Localizations</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Trial Signups</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Video</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Web Content Management</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Whitepaper</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Travel &amp; Accom</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Activations</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>AE Emails</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Chat</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Content Syndication</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Customer Retention &amp; Growth</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Direct Mails</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Direct Traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Display</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>External List Buys</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>In-Product</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Influencer</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Internal Referral</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Organic Search</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Organic Social</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Outbound Prospecting</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Paid Search</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="E56" t="inlineStr">
         <is>
           <t>Paid Media</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Marketing Emails</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
+    <row r="57">
+      <c r="E57" t="inlineStr">
         <is>
           <t>Paid Social</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Marketplace Signups</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
+    <row r="58">
+      <c r="E58" t="inlineStr">
         <is>
           <t>Partner Referral</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Newsletter</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Podcast</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>On-Demand Webinar</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
+    <row r="59">
+      <c r="E59" t="inlineStr">
         <is>
           <t>Press Release</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Other Miscellaneous</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
+    <row r="60">
+      <c r="E60" t="inlineStr">
         <is>
           <t>Print</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Partner Lead Submission</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
+    <row r="61">
+      <c r="E61" t="inlineStr">
         <is>
           <t>Referral Traffic</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Podcast</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
+    <row r="62">
+      <c r="E62" t="inlineStr">
         <is>
           <t>Reseller Registrations</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Presentation</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
+    <row r="63">
+      <c r="E63" t="inlineStr">
         <is>
           <t>Review Site Traffic</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Promotion fee for ISV/Channel Partner</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
+    <row r="64">
+      <c r="E64" t="inlineStr">
         <is>
           <t>SDR Emails</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Reports</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
+    <row r="65">
+      <c r="E65" t="inlineStr">
         <is>
           <t>Support Email</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>ROI Calculator</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
+    <row r="66">
+      <c r="E66" t="inlineStr">
         <is>
           <t>Telemarketing</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Survey</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
+    <row r="67">
+      <c r="E67" t="inlineStr">
         <is>
           <t>Web Publishing</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Translations &amp; Localizations</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Trial Signups</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Video</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Web Content Management</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Whitepaper</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Travel &amp; Accom</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Activations</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Others</t>
         </is>
       </c>
     </row>
@@ -1876,31 +1833,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>How to fill this template</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="200" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Open this file in Microsoft Excel (desktop). Google Sheets, Excel for the web, and Apple Numbers often ignore these dropdowns.
+    <row r="3" ht="240" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Works in Google Sheets: File → Open, or upload to Drive and Open with Google Sheets. Keep the DropdownLists sheet.
 1. Keep the Import sheet headers as they are.
 2. One Type=Campaign row per campaign (Team, Campaign, CampaignType, SubCampaignType, …).
 3. Then one Type=Asset or Type=Tactic row per spend line. Rows link by Campaign name.
-4. Pick CampaignType first — SubCampaignType then only shows related values.
-5. Pick Type = Asset or Tactic — LineName then only shows that list.
+4. SubCampaignType must belong to that row’s CampaignType (import will reject mismatches).
+5. LineName must be an Asset name when Type=Asset, or a Tactic name when Type=Tactic.
 6. Leave LineName blank on Campaign rows.
 7. Delete the example rows before importing real data.
-8. Upload this .xlsx in Data Entry → Bulk import.
+8. Download as Excel (.xlsx) or CSV from Sheets, then upload in Data Entry → Bulk import.
 9. Do not delete the DropdownLists sheet — the dropdowns read from it.
 10. Values are saved as the same text fields as the campaign form.</t>
         </is>
@@ -1917,9 +1874,11 @@
     <row r="12"/>
     <row r="13"/>
     <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A3:A14"/>
+    <mergeCell ref="A3:A16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Tell users Excel desktop has the dropdowns; Google Sheets will not keep them.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/frontend/campaign-import-template.xlsx
+++ b/frontend/campaign-import-template.xlsx
@@ -1849,7 +1849,7 @@
     <row r="3" ht="240" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Works in Google Sheets: File → Open, or upload to Drive and Open with Google Sheets. Keep the DropdownLists sheet.
+          <t>Open this file in Excel on your computer. Dropdown arrows work there. Google Sheets removes Excel dropdowns on convert — in Sheets, Data → Data validation, list from the DropdownLists sheet.
 1. Keep the Import sheet headers as they are.
 2. One Type=Campaign row per campaign (Team, Campaign, CampaignType, SubCampaignType, …).
 3. Then one Type=Asset or Type=Tactic row per spend line. Rows link by Campaign name.
@@ -1857,8 +1857,8 @@
 5. LineName must be an Asset name when Type=Asset, or a Tactic name when Type=Tactic.
 6. Leave LineName blank on Campaign rows.
 7. Delete the example rows before importing real data.
-8. Download as Excel (.xlsx) or CSV from Sheets, then upload in Data Entry → Bulk import.
-9. Do not delete the DropdownLists sheet — the dropdowns read from it.
+8. Upload this .xlsx, or a CSV/xlsx export from Sheets, in Data Entry → Bulk import.
+9. Do not delete the DropdownLists sheet — Excel dropdowns read from it.
 10. Values are saved as the same text fields as the campaign form.</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Update CampaignType/SubCampaignType, Asset, and Tactic taxonomies
Adds Paid Referral and Paid LLM under CampaignType Paid, plus two new
CampaignTypes (Press Release, Others) - matches the current org taxonomy.
Adds Printing/Signage and Speakers to the Asset list, QR Code to the Tactic
list. Updates both the manual entry form's dropdowns (ASSET_TAXONOMY/
TACTIC_TAXONOMY) and the bulk-import validation lists (IMPORT_*) in
frontend/index.html, keeps dashboard-pilot.html byte-identical, and updates
scripts/build_campaign_import_template.py + rebuilds the xlsx template's
DropdownLists sheet so Excel's dropdowns match too.

Also commits backend/step2_finalize.sql (already run against production
earlier - the FK-add + rename-to-legacy2_* step of the DB consolidation),
which hadn't been committed yet.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/campaign-import-template.xlsx
+++ b/frontend/campaign-import-template.xlsx
@@ -1130,16 +1130,16 @@
       <formula1>=DropdownLists!$C$2:$C$4</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Pick a campaign type from the list" promptTitle="Choose from list" prompt="Pick a campaign type" type="list">
-      <formula1>=DropdownLists!$A$2:$A$10</formula1>
+      <formula1>=DropdownLists!$A$2:$A$12</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Pick a sub type from the list" promptTitle="Choose from list" prompt="Must match the CampaignType on this row (checked on import)" type="list">
-      <formula1>=DropdownLists!$D$2:$D$20</formula1>
+      <formula1>=DropdownLists!$D$2:$D$24</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Pick Campaign, Asset, or Tactic" promptTitle="Choose from list" prompt="Campaign (metadata), Asset, or Tactic (spend line)" type="list">
       <formula1>=DropdownLists!$B$2:$B$4</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I500" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid value" error="Pick a LineName from the list" promptTitle="Choose from list" prompt="Assets and tactics. Import rejects a name that does not match Type." type="list">
-      <formula1>=DropdownLists!$E$2:$E$67</formula1>
+      <formula1>=DropdownLists!$E$2:$E$70</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1153,7 +1153,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E67"/>
+  <dimension ref="A1:E70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1374,6 +1374,11 @@
       </c>
     </row>
     <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Press Release</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
           <t>Nurture Campaign</t>
@@ -1386,6 +1391,11 @@
       </c>
     </row>
     <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr">
         <is>
           <t>Paid Search</t>
@@ -1424,7 +1434,7 @@
     <row r="15">
       <c r="D15" t="inlineStr">
         <is>
-          <t>Organic Social</t>
+          <t>Paid Referral</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1436,7 +1446,7 @@
     <row r="16">
       <c r="D16" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Paid LLM</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1448,7 +1458,7 @@
     <row r="17">
       <c r="D17" t="inlineStr">
         <is>
-          <t>Content Syndication</t>
+          <t>Organic Social</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1460,7 +1470,7 @@
     <row r="18">
       <c r="D18" t="inlineStr">
         <is>
-          <t>Demo Request</t>
+          <t>Organic Search</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1472,7 +1482,7 @@
     <row r="19">
       <c r="D19" t="inlineStr">
         <is>
-          <t>Referral Traffic</t>
+          <t>Content Syndication</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1484,23 +1494,33 @@
     <row r="20">
       <c r="D20" t="inlineStr">
         <is>
+          <t>Demo Request</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Landing Page Copy</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Referral Traffic</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Marketing Emails</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="D22" t="inlineStr">
+        <is>
           <t>Direct Mail</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Landing Page Copy</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Marketing Emails</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
       <c r="E22" t="inlineStr">
         <is>
           <t>Marketplace Signups</t>
@@ -1508,6 +1528,11 @@
       </c>
     </row>
     <row r="23">
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Press Release</t>
+        </is>
+      </c>
       <c r="E23" t="inlineStr">
         <is>
           <t>Newsletter</t>
@@ -1515,6 +1540,11 @@
       </c>
     </row>
     <row r="24">
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
       <c r="E24" t="inlineStr">
         <is>
           <t>On-Demand Webinar</t>
@@ -1636,189 +1666,210 @@
     <row r="41">
       <c r="E41" t="inlineStr">
         <is>
-          <t>AE Emails</t>
+          <t>Printing/Signage</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="E42" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Speakers</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="E43" t="inlineStr">
         <is>
-          <t>Content Syndication</t>
+          <t>AE Emails</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="E44" t="inlineStr">
         <is>
-          <t>Customer Retention &amp; Growth</t>
+          <t>Chat</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="E45" t="inlineStr">
         <is>
-          <t>Direct Mails</t>
+          <t>Content Syndication</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="E46" t="inlineStr">
         <is>
-          <t>Direct Traffic</t>
+          <t>Customer Retention &amp; Growth</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="E47" t="inlineStr">
         <is>
-          <t>Display</t>
+          <t>Direct Mails</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="E48" t="inlineStr">
         <is>
-          <t>External List Buys</t>
+          <t>Direct Traffic</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="E49" t="inlineStr">
         <is>
-          <t>In-Product</t>
+          <t>Display</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="E50" t="inlineStr">
         <is>
-          <t>Influencer</t>
+          <t>External List Buys</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="E51" t="inlineStr">
         <is>
-          <t>Internal Referral</t>
+          <t>In-Product</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="E52" t="inlineStr">
         <is>
-          <t>Organic Search</t>
+          <t>Influencer</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="E53" t="inlineStr">
         <is>
-          <t>Organic Social</t>
+          <t>Internal Referral</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="E54" t="inlineStr">
         <is>
-          <t>Outbound Prospecting</t>
+          <t>Organic Search</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="E55" t="inlineStr">
         <is>
-          <t>Paid Search</t>
+          <t>Organic Social</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="E56" t="inlineStr">
         <is>
-          <t>Paid Media</t>
+          <t>Outbound Prospecting</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="E57" t="inlineStr">
         <is>
-          <t>Paid Social</t>
+          <t>Paid Search</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="E58" t="inlineStr">
         <is>
-          <t>Partner Referral</t>
+          <t>Paid Media</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="E59" t="inlineStr">
         <is>
-          <t>Press Release</t>
+          <t>Paid Social</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="E60" t="inlineStr">
         <is>
-          <t>Print</t>
+          <t>Partner Referral</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="E61" t="inlineStr">
         <is>
-          <t>Referral Traffic</t>
+          <t>Press Release</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="E62" t="inlineStr">
         <is>
-          <t>Reseller Registrations</t>
+          <t>Print</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="E63" t="inlineStr">
         <is>
-          <t>Review Site Traffic</t>
+          <t>Referral Traffic</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="E64" t="inlineStr">
         <is>
-          <t>SDR Emails</t>
+          <t>Reseller Registrations</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="E65" t="inlineStr">
         <is>
-          <t>Support Email</t>
+          <t>Review Site Traffic</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="E66" t="inlineStr">
         <is>
-          <t>Telemarketing</t>
+          <t>SDR Emails</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="E67" t="inlineStr">
         <is>
+          <t>Support Email</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Telemarketing</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="E69" t="inlineStr">
+        <is>
           <t>Web Publishing</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>QR Code</t>
         </is>
       </c>
     </row>

</xml_diff>